<commit_message>
finish visualizations for online meeting aug 26
</commit_message>
<xml_diff>
--- a/outputs/coding-answers-human/testList_answers_df_studyResults_v9_human.xlsx
+++ b/outputs/coding-answers-human/testList_answers_df_studyResults_v9_human.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\deviv\R-working-folder\ORO-product-4-R\outputs\coding-anwers-human\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\deviv\R-working-folder\ORO-product-4-R\outputs\coding-answers-human\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="93">
   <si>
     <t>id</t>
   </si>
@@ -248,6 +248,57 @@
   </si>
   <si>
     <t>implementation of the Na tional Climate Change Policy and mainstreaming of climate change mitigation and adaptation responses in coastal sectors has not been as effective as needed. S</t>
+  </si>
+  <si>
+    <t>oro_type</t>
+  </si>
+  <si>
+    <t>['Fisheries management']</t>
+  </si>
+  <si>
+    <t>['Institutional','Economic', 'Socio-behavioural', 'Built infrastructure', 'Nature-based']</t>
+  </si>
+  <si>
+    <t>['Institutional']</t>
+  </si>
+  <si>
+    <t>['Institutional', 'Economic']</t>
+  </si>
+  <si>
+    <t>['Built infrastructure', 'Economic']</t>
+  </si>
+  <si>
+    <t>['Institutional', 'Socio-behavioural', 'Fishing technologies', 'Built infrastructure']</t>
+  </si>
+  <si>
+    <t>['Socio-behavioural', 'Economic', 'Fisheries management']</t>
+  </si>
+  <si>
+    <t>['Socio-behavioural', 'Institutional']</t>
+  </si>
+  <si>
+    <t>['Fisheries management', 'Socio-behavioural', 'Institutional', 'Economic', 'Built infrastructure', 'Nature-based']</t>
+  </si>
+  <si>
+    <t>['Socio-behavioural','Fisheries management','Economic', 'Fishing technologies', 'Built infrastructure']</t>
+  </si>
+  <si>
+    <t>['Socio-behavioural', 'Institutional','Fisheries management', 'Fishing technologies']</t>
+  </si>
+  <si>
+    <t>['Socio-behavioural']</t>
+  </si>
+  <si>
+    <t>['Socio-behavioural', 'Disaster response technologies', 'Built infrastructure', 'Nature-based']</t>
+  </si>
+  <si>
+    <t>['Institutional','Economic', 'Fishing technologies']</t>
+  </si>
+  <si>
+    <t>['Institutional','Fisheries management', 'Disaster response technologies', 'Nature-based']</t>
+  </si>
+  <si>
+    <t>['Fisheries management', 'Institutional']</t>
   </si>
 </sst>
 </file>
@@ -308,7 +359,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -320,6 +371,12 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -622,745 +679,844 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="3" max="3" width="8.7265625" style="6"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>71</v>
       </c>
       <c r="B2" t="s">
         <v>49</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="C2" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="G2" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>85</v>
       </c>
       <c r="B3" t="s">
         <v>49</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="D3" t="s">
         <v>41</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>42</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>10</v>
       </c>
-      <c r="F3" t="s">
-        <v>13</v>
-      </c>
       <c r="G3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" t="s">
         <v>7</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>85</v>
       </c>
       <c r="B4" t="s">
         <v>49</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="D4" t="s">
         <v>43</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>44</v>
       </c>
-      <c r="E4" t="s">
-        <v>9</v>
-      </c>
       <c r="F4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" t="s">
         <v>21</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>7</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>85</v>
       </c>
       <c r="B5" t="s">
         <v>49</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D5" t="s">
         <v>45</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>42</v>
       </c>
-      <c r="E5" t="s">
-        <v>9</v>
-      </c>
       <c r="F5" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G5" t="s">
+        <v>13</v>
+      </c>
+      <c r="H5" t="s">
         <v>7</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>252</v>
       </c>
       <c r="B6" t="s">
         <v>49</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="D6" t="s">
         <v>11</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>50</v>
       </c>
-      <c r="E6" t="s">
-        <v>9</v>
-      </c>
       <c r="F6" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G6" t="s">
+        <v>13</v>
+      </c>
+      <c r="H6" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>283</v>
       </c>
       <c r="B7" t="s">
         <v>49</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="D7" t="s">
         <v>17</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>12</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>18</v>
       </c>
-      <c r="F7" t="s">
-        <v>13</v>
-      </c>
       <c r="G7" t="s">
+        <v>13</v>
+      </c>
+      <c r="H7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>283</v>
       </c>
       <c r="B8" t="s">
         <v>49</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="D8" t="s">
         <v>51</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>12</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>18</v>
       </c>
-      <c r="F8" t="s">
-        <v>13</v>
-      </c>
       <c r="G8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H8" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>293</v>
       </c>
       <c r="B9" t="s">
         <v>49</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="D9" t="s">
         <v>52</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>19</v>
       </c>
-      <c r="E9" t="s">
-        <v>9</v>
-      </c>
       <c r="F9" t="s">
+        <v>9</v>
+      </c>
+      <c r="G9" t="s">
         <v>21</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>293</v>
       </c>
       <c r="B10" t="s">
         <v>49</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="D10" t="s">
         <v>52</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>19</v>
       </c>
-      <c r="E10" t="s">
-        <v>9</v>
-      </c>
       <c r="F10" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G10" t="s">
+        <v>13</v>
+      </c>
+      <c r="H10" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>480</v>
       </c>
       <c r="B11" t="s">
         <v>49</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="D11" t="s">
         <v>53</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>12</v>
       </c>
-      <c r="E11" t="s">
-        <v>9</v>
-      </c>
       <c r="F11" t="s">
+        <v>9</v>
+      </c>
+      <c r="G11" t="s">
         <v>21</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A12" s="4">
         <v>538</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="D12" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="E12" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E12" s="4" t="s">
-        <v>9</v>
-      </c>
       <c r="F12" s="4" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G12" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H12" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="H12" s="4" t="s">
+      <c r="I12" s="4" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>1678</v>
       </c>
       <c r="B13" t="s">
         <v>49</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="D13" t="s">
         <v>56</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>19</v>
       </c>
-      <c r="E13" t="s">
+      <c r="F13" t="s">
         <v>18</v>
       </c>
-      <c r="F13" t="s">
-        <v>13</v>
-      </c>
       <c r="G13" t="s">
+        <v>13</v>
+      </c>
+      <c r="H13" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>1678</v>
       </c>
       <c r="B14" t="s">
         <v>49</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="D14" t="s">
         <v>57</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
         <v>25</v>
       </c>
-      <c r="E14" t="s">
+      <c r="F14" t="s">
         <v>18</v>
       </c>
-      <c r="F14" t="s">
+      <c r="G14" t="s">
         <v>21</v>
       </c>
-      <c r="G14" t="s">
+      <c r="H14" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>5078</v>
       </c>
       <c r="B15" t="s">
         <v>49</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="D15" t="s">
         <v>59</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
         <v>58</v>
       </c>
-      <c r="E15" t="s">
+      <c r="F15" t="s">
         <v>18</v>
       </c>
-      <c r="F15" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="G15" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>5078</v>
       </c>
       <c r="B16" t="s">
         <v>49</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="D16" t="s">
         <v>60</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>19</v>
       </c>
-      <c r="E16" t="s">
-        <v>9</v>
-      </c>
       <c r="F16" t="s">
+        <v>9</v>
+      </c>
+      <c r="G16" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>5171</v>
       </c>
       <c r="B17" t="s">
         <v>49</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="D17" t="s">
         <v>61</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>19</v>
       </c>
-      <c r="E17" t="s">
-        <v>9</v>
-      </c>
       <c r="F17" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+        <v>9</v>
+      </c>
+      <c r="G17" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>5171</v>
       </c>
       <c r="B18" t="s">
         <v>49</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="D18" t="s">
         <v>62</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>19</v>
       </c>
-      <c r="E18" t="s">
-        <v>9</v>
-      </c>
       <c r="F18" t="s">
+        <v>9</v>
+      </c>
+      <c r="G18" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>5171</v>
       </c>
       <c r="B19" t="s">
         <v>49</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="D19" t="s">
         <v>63</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
         <v>15</v>
       </c>
-      <c r="E19" t="s">
-        <v>9</v>
-      </c>
       <c r="F19" t="s">
+        <v>9</v>
+      </c>
+      <c r="G19" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>5281</v>
       </c>
       <c r="B20" t="s">
         <v>49</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="D20" t="s">
         <v>46</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E20" t="s">
         <v>64</v>
       </c>
-      <c r="E20" t="s">
-        <v>9</v>
-      </c>
       <c r="F20" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G20" t="s">
+        <v>13</v>
+      </c>
+      <c r="H20" t="s">
         <v>27</v>
       </c>
-      <c r="H20" t="s">
+      <c r="I20" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>5281</v>
       </c>
       <c r="B21" t="s">
         <v>49</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="D21" t="s">
         <v>65</v>
       </c>
-      <c r="D21" t="s">
+      <c r="E21" t="s">
         <v>12</v>
       </c>
-      <c r="E21" t="s">
+      <c r="F21" t="s">
         <v>18</v>
       </c>
-      <c r="F21" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="G21" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>6502</v>
       </c>
       <c r="B22" t="s">
         <v>49</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="D22" t="s">
         <v>66</v>
       </c>
-      <c r="D22" t="s">
+      <c r="E22" t="s">
         <v>47</v>
       </c>
-      <c r="E22" t="s">
+      <c r="F22" t="s">
         <v>18</v>
       </c>
-      <c r="F22" t="s">
+      <c r="G22" t="s">
         <v>21</v>
       </c>
-      <c r="G22" t="s">
+      <c r="H22" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>8058</v>
       </c>
       <c r="B23" t="s">
         <v>49</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="D23" t="s">
         <v>10</v>
       </c>
-      <c r="D23" t="s">
+      <c r="E23" t="s">
         <v>34</v>
       </c>
-      <c r="E23" t="s">
-        <v>9</v>
-      </c>
       <c r="F23" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G23" t="s">
+        <v>13</v>
+      </c>
+      <c r="H23" t="s">
         <v>30</v>
       </c>
-      <c r="H23" t="s">
+      <c r="I23" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>10064</v>
       </c>
       <c r="B24" t="s">
         <v>49</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="D24" t="s">
         <v>67</v>
       </c>
-      <c r="D24" t="s">
+      <c r="E24" t="s">
         <v>12</v>
       </c>
-      <c r="E24" t="s">
+      <c r="F24" t="s">
         <v>18</v>
       </c>
-      <c r="F24" t="s">
+      <c r="G24" t="s">
         <v>21</v>
       </c>
-      <c r="G24" t="s">
+      <c r="H24" t="s">
         <v>32</v>
       </c>
-      <c r="H24" t="s">
+      <c r="I24" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>232677</v>
       </c>
       <c r="B25" t="s">
         <v>49</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="D25" t="s">
         <v>69</v>
       </c>
-      <c r="D25" t="s">
+      <c r="E25" t="s">
         <v>19</v>
       </c>
-      <c r="E25" t="s">
-        <v>9</v>
-      </c>
       <c r="F25" t="s">
+        <v>9</v>
+      </c>
+      <c r="G25" t="s">
         <v>21</v>
       </c>
-      <c r="G25" t="s">
+      <c r="H25" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>232677</v>
       </c>
       <c r="B26" t="s">
         <v>49</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="D26" t="s">
         <v>68</v>
       </c>
-      <c r="D26" t="s">
+      <c r="E26" t="s">
         <v>70</v>
       </c>
-      <c r="E26" t="s">
-        <v>9</v>
-      </c>
       <c r="F26" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G26" t="s">
+        <v>13</v>
+      </c>
+      <c r="H26" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>244602</v>
       </c>
       <c r="B27" t="s">
         <v>49</v>
       </c>
-      <c r="D27" t="s">
+      <c r="C27" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="E27" t="s">
         <v>19</v>
       </c>
-      <c r="E27" t="s">
+      <c r="F27" t="s">
         <v>18</v>
       </c>
-      <c r="F27" t="s">
-        <v>13</v>
-      </c>
       <c r="G27" t="s">
+        <v>13</v>
+      </c>
+      <c r="H27" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>249273</v>
       </c>
       <c r="B28" t="s">
         <v>49</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C28" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="D28" t="s">
         <v>71</v>
       </c>
-      <c r="D28" t="s">
+      <c r="E28" t="s">
         <v>19</v>
       </c>
-      <c r="E28" t="s">
-        <v>9</v>
-      </c>
       <c r="F28" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G28" t="s">
+        <v>13</v>
+      </c>
+      <c r="H28" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>249273</v>
       </c>
       <c r="B29" t="s">
         <v>49</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C29" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="D29" t="s">
         <v>72</v>
       </c>
-      <c r="D29" t="s">
+      <c r="E29" t="s">
         <v>19</v>
       </c>
-      <c r="E29" t="s">
-        <v>9</v>
-      </c>
       <c r="F29" t="s">
+        <v>9</v>
+      </c>
+      <c r="G29" t="s">
         <v>21</v>
       </c>
-      <c r="G29" t="s">
+      <c r="H29" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>250635</v>
       </c>
       <c r="B30" t="s">
         <v>49</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C30" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="D30" t="s">
         <v>73</v>
       </c>
-      <c r="D30" t="s">
+      <c r="E30" t="s">
         <v>19</v>
       </c>
-      <c r="E30" t="s">
-        <v>9</v>
-      </c>
       <c r="F30" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G30" t="s">
+        <v>13</v>
+      </c>
+      <c r="H30" t="s">
         <v>38</v>
       </c>
-      <c r="H30" t="s">
+      <c r="I30" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>250635</v>
       </c>
       <c r="B31" t="s">
         <v>49</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C31" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="D31" t="s">
         <v>74</v>
       </c>
-      <c r="D31" t="s">
+      <c r="E31" t="s">
         <v>19</v>
       </c>
-      <c r="E31" t="s">
-        <v>9</v>
-      </c>
       <c r="F31" t="s">
+        <v>9</v>
+      </c>
+      <c r="G31" t="s">
         <v>21</v>
       </c>
-      <c r="G31" t="s">
+      <c r="H31" t="s">
         <v>38</v>
       </c>
-      <c r="H31" t="s">
+      <c r="I31" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>259944</v>
       </c>
       <c r="B32" t="s">
         <v>49</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C32" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="D32" t="s">
         <v>75</v>
       </c>
-      <c r="D32" t="s">
+      <c r="E32" t="s">
         <v>19</v>
       </c>
-      <c r="E32" t="s">
-        <v>9</v>
-      </c>
       <c r="F32" t="s">
+        <v>9</v>
+      </c>
+      <c r="G32" t="s">
         <v>21</v>
       </c>
-      <c r="G32" t="s">
+      <c r="H32" t="s">
         <v>40</v>
       </c>
     </row>

</xml_diff>